<commit_message>
回退代码至 2.5.15 版本 (57d7995)
将代码库整体恢复至提交 57d7995dfe（CM Schema update to 2.5.15）的状态。

Co-authored-by: eatsleepractice <eatsleepractice0@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mes-plugins/mes-plugins-basic/src/main/resources/basic/public/resources/productImportSchema_cn.xlsx
+++ b/mes-plugins/mes-plugins-basic/src/main/resources/basic/public/resources/productImportSchema_cn.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/krna/Projects/mes/mes-plugins/mes-plugins-basic/src/main/resources/basic/public/resources/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pdutka\Desktop\Import templates - 副本\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC920048-93FE-664A-AE17-224AE3C29306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F4BE8E-5A67-4DB4-81F3-AE066EB19316}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -63,7 +62,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -88,7 +86,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -97,7 +94,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -117,7 +113,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -131,7 +126,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -140,7 +134,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -160,7 +153,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -179,7 +171,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">:
 - </t>
@@ -199,7 +190,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">,
 - </t>
@@ -219,7 +209,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">,
 - </t>
@@ -239,7 +228,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">, 
 - </t>
@@ -259,7 +247,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">,
 - </t>
@@ -279,7 +266,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -293,7 +279,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -302,7 +287,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -322,7 +306,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -346,7 +329,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -355,7 +337,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -375,7 +356,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -394,7 +374,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve"> </t>
         </r>
@@ -418,7 +397,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -427,7 +405,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -447,7 +424,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -466,7 +442,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -486,7 +461,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>:</t>
         </r>
@@ -505,7 +479,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>“box”</t>
         </r>
@@ -524,7 +497,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>“pcs”</t>
         </r>
@@ -543,7 +515,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>10</t>
         </r>
@@ -562,7 +533,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>= 10</t>
         </r>
@@ -586,7 +556,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -595,7 +564,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -615,7 +583,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -634,7 +601,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>EAN</t>
         </r>
@@ -653,7 +619,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>:</t>
         </r>
@@ -672,7 +637,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>EAN</t>
         </r>
@@ -696,7 +660,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -705,7 +668,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -725,7 +687,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -749,7 +710,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -758,7 +718,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -778,7 +737,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -792,7 +750,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -801,7 +758,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -821,7 +777,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -845,7 +800,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -854,7 +808,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -874,7 +827,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -893,7 +845,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -907,7 +858,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -916,7 +866,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -936,7 +885,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -955,7 +903,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo</t>
         </r>
@@ -979,7 +926,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -988,7 +934,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -1008,7 +953,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>5</t>
         </r>
@@ -1027,7 +971,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>0.12345</t>
         </r>
@@ -1041,7 +984,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -1050,7 +992,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -1070,7 +1011,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>5</t>
         </r>
@@ -1089,7 +1029,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>0.12345</t>
         </r>
@@ -1103,7 +1042,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -1112,7 +1050,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -1132,7 +1069,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>5</t>
         </r>
@@ -1151,7 +1087,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>0.12345</t>
         </r>
@@ -1165,7 +1100,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -1174,7 +1108,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -1194,7 +1127,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>.</t>
         </r>
@@ -1208,7 +1140,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -1217,7 +1148,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -1242,7 +1172,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>qcadoo MES:</t>
         </r>
@@ -1251,7 +1180,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 </t>
@@ -1271,7 +1199,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">. </t>
         </r>
@@ -1290,7 +1217,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve"> '</t>
         </r>
@@ -1309,7 +1235,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve">' </t>
         </r>
@@ -1328,7 +1253,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t xml:space="preserve"> '</t>
         </r>
@@ -1347,7 +1271,6 @@
             <sz val="11"/>
             <color indexed="8"/>
             <rFont val="Helvetica Neue"/>
-            <family val="2"/>
           </rPr>
           <t>'.</t>
         </r>
@@ -1358,7 +1281,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Y/N</t>
   </si>
@@ -1476,9 +1399,6 @@
   <si>
     <t>包装品</t>
   </si>
-  <si>
-    <t>Expiration date evidence</t>
-  </si>
 </sst>
 </file>
 
@@ -1520,13 +1440,11 @@
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1620,28 +1538,9 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <charset val="238"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
+  <dxfs count="21">
     <dxf>
       <font>
         <b val="0"/>
@@ -2047,7 +1946,7 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Styl tabeli 1" pivot="0" count="1" xr9:uid="{5916ACAE-860C-41DE-93CE-65C632F1090D}">
-      <tableStyleElement type="wholeTable" dxfId="21"/>
+      <tableStyleElement type="wholeTable" dxfId="20"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2704,28 +2603,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3EF1E979-207E-47C4-9AFE-5BA280F7BEEC}" name="productImportSchema_en" displayName="productImportSchema_en" ref="A1:S2" insertRow="1" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
-  <autoFilter ref="A1:S2" xr:uid="{3EF1E979-207E-47C4-9AFE-5BA280F7BEEC}"/>
-  <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{2C201668-3CD6-489F-809C-EFB4F2E697A6}" name="产品编号" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{BED42B7C-AA1C-4D86-A97D-42DFF2ABFC99}" name="产品名称" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{2BD0676B-09A5-4D52-8D38-762C5FC845F5}" name="物料类型" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{C478A5DE-164D-4B5E-B227-B82363809398}" name="默认单位" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{3ECE3C08-28FA-455A-809D-5D8C51C53951}" name="附加单位" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{D6356E1B-1498-4F42-8E53-B5E002D3ADD8}" name="单位换算" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{F93F6B18-4CC2-4826-8065-0BAC652D8244}" name="EAN 编码" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{F57ED3FB-C444-4D0D-9912-DFCBFC297B8C}" name="种类" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{F16578D4-258B-4578-BE1C-484CCC898684}" name="描述" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{483CFD25-B432-4F34-9C86-0D60BA26D995}" name="制造商" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{CD301045-E17B-4F44-A794-67E6CBA37A43}" name="分类" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{F8FE13EF-6730-42F0-92D7-8A2A9C0F0F90}" name="所属系列" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{EC10C708-462E-42D9-9789-115BB59EC60F}" name="名义成本" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{20E3562B-134E-4CEC-8D4B-FA4A24FAB1C9}" name="最新采购成本" dataDxfId="5"/>
-    <tableColumn id="15" xr3:uid="{B9A08066-9499-46BD-B4BA-457BB4EB7E4A}" name="平均成本" dataDxfId="4"/>
-    <tableColumn id="16" xr3:uid="{BA516DDF-89CD-4830-8234-28B7361601F4}" name="尺寸" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{2E84D04E-647F-4253-8983-F87E0652FDD8}" name="有效期" dataDxfId="2"/>
-    <tableColumn id="18" xr3:uid="{E00DEA52-A691-460C-978D-6D41BD23C0AF}" name="批次依据" dataDxfId="1"/>
-    <tableColumn id="19" xr3:uid="{48A8DDB9-8367-1845-AFE8-B6352E32B5F5}" name="Expiration date evidence" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3EF1E979-207E-47C4-9AFE-5BA280F7BEEC}" name="productImportSchema_en" displayName="productImportSchema_en" ref="A1:R2" insertRow="1" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+  <autoFilter ref="A1:R2" xr:uid="{3EF1E979-207E-47C4-9AFE-5BA280F7BEEC}"/>
+  <tableColumns count="18">
+    <tableColumn id="1" xr3:uid="{2C201668-3CD6-489F-809C-EFB4F2E697A6}" name="产品编号" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{BED42B7C-AA1C-4D86-A97D-42DFF2ABFC99}" name="产品名称" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{2BD0676B-09A5-4D52-8D38-762C5FC845F5}" name="物料类型" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{C478A5DE-164D-4B5E-B227-B82363809398}" name="默认单位" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{3ECE3C08-28FA-455A-809D-5D8C51C53951}" name="附加单位" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{D6356E1B-1498-4F42-8E53-B5E002D3ADD8}" name="单位换算" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{F93F6B18-4CC2-4826-8065-0BAC652D8244}" name="EAN 编码" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{F57ED3FB-C444-4D0D-9912-DFCBFC297B8C}" name="种类" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{F16578D4-258B-4578-BE1C-484CCC898684}" name="描述" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{483CFD25-B432-4F34-9C86-0D60BA26D995}" name="制造商" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{CD301045-E17B-4F44-A794-67E6CBA37A43}" name="分类" dataDxfId="7"/>
+    <tableColumn id="12" xr3:uid="{F8FE13EF-6730-42F0-92D7-8A2A9C0F0F90}" name="所属系列" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{EC10C708-462E-42D9-9789-115BB59EC60F}" name="名义成本" dataDxfId="5"/>
+    <tableColumn id="14" xr3:uid="{20E3562B-134E-4CEC-8D4B-FA4A24FAB1C9}" name="最新采购成本" dataDxfId="4"/>
+    <tableColumn id="15" xr3:uid="{B9A08066-9499-46BD-B4BA-457BB4EB7E4A}" name="平均成本" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{BA516DDF-89CD-4830-8234-28B7361601F4}" name="尺寸" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{2E84D04E-647F-4253-8983-F87E0652FDD8}" name="有效期" dataDxfId="1"/>
+    <tableColumn id="18" xr3:uid="{E00DEA52-A691-460C-978D-6D41BD23C0AF}" name="批次依据" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="Styl tabeli 1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2752,9 +2650,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office 2013–2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Pakiet Office 2013–2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2792,7 +2690,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Pakiet Office 2013–2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2898,7 +2796,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Pakiet Office 2013–2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3040,7 +2938,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3051,20 +2949,20 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="2" width="16.83203125" style="1" customWidth="1"/>
+    <col min="1" max="2" width="16.875" style="1" customWidth="1"/>
     <col min="3" max="3" width="22.5" style="1" customWidth="1"/>
-    <col min="4" max="5" width="20.83203125" style="1" customWidth="1"/>
-    <col min="6" max="11" width="16.83203125" style="1" customWidth="1"/>
+    <col min="4" max="5" width="20.875" style="1" customWidth="1"/>
+    <col min="6" max="11" width="16.875" style="1" customWidth="1"/>
     <col min="12" max="12" width="17.5" style="1" customWidth="1"/>
-    <col min="13" max="15" width="20.83203125" style="1" customWidth="1"/>
-    <col min="16" max="18" width="16.83203125" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.83203125" style="1"/>
+    <col min="13" max="15" width="20.875" style="1" customWidth="1"/>
+    <col min="16" max="18" width="16.875" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:18">
       <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
@@ -3119,11 +3017,8 @@
       <c r="R1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:18">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="D2" s="2"/>
@@ -3168,7 +3063,7 @@
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="22.5" customWidth="1"/>
   </cols>

</xml_diff>